<commit_message>
implements most of #2227 and #2228
</commit_message>
<xml_diff>
--- a/data/translations.wikidata.xlsx
+++ b/data/translations.wikidata.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -34,16 +34,28 @@
     <t xml:space="preserve">English</t>
   </si>
   <si>
+    <t xml:space="preserve">id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">de</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">en</t>
+  </si>
+  <si>
     <t xml:space="preserve">filter_ref</t>
   </si>
   <si>
-    <t xml:space="preserve">Normdatenbank</t>
+    <t xml:space="preserve">Datenbank</t>
   </si>
   <si>
     <t xml:space="preserve">refs</t>
   </si>
   <si>
-    <t xml:space="preserve">Normdatenbanken</t>
+    <t xml:space="preserve">Datenbanken</t>
   </si>
   <si>
     <t xml:space="preserve">or</t>
@@ -68,6 +80,36 @@
   </si>
   <si>
     <t xml:space="preserve">Wikdata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">results</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resultate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">result</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resultat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">search_prompt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Freitextsuche Namen oder Nummer des Wikidata Items</t>
+  </si>
+  <si>
+    <t xml:space="preserve">selection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auswahl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no_reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nicht referenziert</t>
   </si>
 </sst>
 </file>
@@ -209,48 +251,101 @@
       <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="C2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="1048505" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
     <row r="1048506" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048507" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048508" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>